<commit_message>
added 2026 round 2 results
</commit_message>
<xml_diff>
--- a/bio/player_bio.xlsx
+++ b/bio/player_bio.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/matevass/Documents/Programming/R/darts-statistics/bio/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E63ACEE-AE81-F24D-9D53-DAF683CFD428}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48C6512D-1D3C-E349-AC48-668CCB0CE9EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="20020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -177,9 +177,6 @@
     <t>23g Red Dragon Fury 2</t>
   </si>
   <si>
-    <t>21g Bulls</t>
-  </si>
-  <si>
     <t>Geri Vass</t>
   </si>
   <si>
@@ -232,6 +229,9 @@
   </si>
   <si>
     <t>23g Red Dragon Rebel</t>
+  </si>
+  <si>
+    <t>21.5g Winmau MvG ExAct</t>
   </si>
 </sst>
 </file>
@@ -711,7 +711,7 @@
         <v>46</v>
       </c>
       <c r="H4" s="6">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -719,7 +719,7 @@
         <v>17</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>18</v>
@@ -734,7 +734,7 @@
         <v>9</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="H5" s="6">
         <v>11</v>
@@ -812,10 +812,10 @@
         <v>9</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="H8" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -864,7 +864,7 @@
         <v>9</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>48</v>
+        <v>66</v>
       </c>
       <c r="H10" s="6">
         <v>1</v>
@@ -890,7 +890,7 @@
         <v>9</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="H11" s="6">
         <v>0</v>
@@ -916,7 +916,7 @@
         <v>9</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="H12" s="6">
         <v>0</v>
@@ -924,13 +924,13 @@
     </row>
     <row r="13" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A13" s="6" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C13" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D13" s="3">
         <v>37437</v>
@@ -942,7 +942,7 @@
         <v>9</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="H13" s="6">
         <v>0</v>
@@ -950,13 +950,13 @@
     </row>
     <row r="14" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A14" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="B14" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="C14" t="s">
         <v>50</v>
-      </c>
-      <c r="B14" s="9" t="s">
-        <v>52</v>
-      </c>
-      <c r="C14" t="s">
-        <v>51</v>
       </c>
       <c r="D14" s="3">
         <v>36552</v>
@@ -968,7 +968,7 @@
         <v>9</v>
       </c>
       <c r="G14" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="H14" s="6">
         <v>0</v>
@@ -976,13 +976,13 @@
     </row>
     <row r="15" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A15" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="B15" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="B15" s="9" t="s">
+      <c r="C15" t="s">
         <v>58</v>
-      </c>
-      <c r="C15" t="s">
-        <v>59</v>
       </c>
       <c r="D15" s="3">
         <v>39597</v>
@@ -994,7 +994,7 @@
         <v>9</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="H15" s="6">
         <v>2</v>
@@ -1002,13 +1002,13 @@
     </row>
     <row r="16" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A16" s="10" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B16" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="C16" s="8" t="s">
         <v>61</v>
-      </c>
-      <c r="C16" s="8" t="s">
-        <v>62</v>
       </c>
       <c r="D16" s="13">
         <v>36412</v>
@@ -1020,7 +1020,7 @@
         <v>9</v>
       </c>
       <c r="G16" s="8" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="H16" s="12">
         <v>5</v>

</xml_diff>

<commit_message>
added 2026 round 3 results
</commit_message>
<xml_diff>
--- a/bio/player_bio.xlsx
+++ b/bio/player_bio.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/matevass/Documents/Programming/R/darts-statistics/bio/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E22F5F0A-FFDF-7E42-932E-B7A8B7DB5A38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B1F70B7-ECF1-214A-AE66-FD855898A7AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="20020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="68">
   <si>
     <t>Player</t>
   </si>
@@ -232,6 +232,9 @@
   </si>
   <si>
     <t>24g Red Dragon Seren 3 Onyx</t>
+  </si>
+  <si>
+    <t>22g Winmau MvG Assault</t>
   </si>
 </sst>
 </file>
@@ -667,7 +670,7 @@
         <v>10</v>
       </c>
       <c r="H2" s="6">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -976,7 +979,7 @@
         <v>9</v>
       </c>
       <c r="G14" t="s">
-        <v>53</v>
+        <v>67</v>
       </c>
       <c r="H14" s="6">
         <v>0</v>

</xml_diff>

<commit_message>
added 2026 round 4 results
</commit_message>
<xml_diff>
--- a/bio/player_bio.xlsx
+++ b/bio/player_bio.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/matevass/Documents/Programming/R/darts-statistics/bio/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B1F70B7-ECF1-214A-AE66-FD855898A7AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7881D9BD-5516-D64D-BA4A-39F700ACF160}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="20020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="16420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -748,7 +748,7 @@
         <v>62</v>
       </c>
       <c r="H5" s="6">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -1034,7 +1034,7 @@
         <v>66</v>
       </c>
       <c r="H16" s="12">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>